<commit_message>
image backend storage added
</commit_message>
<xml_diff>
--- a/next-dashboard-ui/attendance_cctv/backend/exports/attendance_star_2026_04.xlsx
+++ b/next-dashboard-ui/attendance_cctv/backend/exports/attendance_star_2026_04.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH5"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -883,7 +883,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -972,23 +972,23 @@
         </is>
       </c>
       <c r="AG3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vorta</t>
+          <t>Rafia Tasnim</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>P</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1142,23 +1142,23 @@
         </is>
       </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>3.33%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zara Rahman</t>
+          <t>Vorta</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1317,6 +1317,176 @@
       <c r="AH5" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Zara Rahman</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AG6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>3.33%</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1387,39 +1557,39 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>10.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vorta</t>
+          <t>Rafia Tasnim</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>3.33%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zara Rahman</t>
+          <t>Vorta</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1431,6 +1601,24 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Zara Rahman</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3.33%</t>
         </is>
       </c>
     </row>

</xml_diff>